<commit_message>
admin puede crear mas admins, y agregue imagenes al excel
</commit_message>
<xml_diff>
--- a/Documentacion/Casos de Prueba.xlsx
+++ b/Documentacion/Casos de Prueba.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leona\OneDrive\Escritorio\TAG-OK\Documentacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\igna_\OneDrive\Documentos\Tag OK\TAG-OK\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{538B0C3B-56AB-4547-8D9C-8D21FBAD9C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42227A0E-D434-408F-879A-5BDFE387F527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Suite de pruebas" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,78 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="6">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="6">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+  </valueMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -390,6 +462,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -398,14 +476,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,6 +936,95 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+</richValueRels>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -1063,33 +1224,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z66"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" customWidth="1"/>
     <col min="4" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="26.109375" customWidth="1"/>
-    <col min="7" max="7" width="17.109375" customWidth="1"/>
-    <col min="8" max="8" width="127.6640625" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.140625" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="127.7109375" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" customWidth="1"/>
-    <col min="11" max="26" width="10.88671875" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" customWidth="1"/>
+    <col min="11" max="26" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="14"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -1110,7 +1271,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1158,18 +1319,18 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="14"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -1188,7 +1349,7 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" ht="274.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" ht="274.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="5" t="s">
         <v>12</v>
@@ -1230,7 +1391,7 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="282.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" ht="282.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="5" t="s">
         <v>18</v>
@@ -1271,17 +1432,17 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -1301,7 +1462,7 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="216.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="5" t="s">
         <v>23</v>
@@ -1309,7 +1470,7 @@
       <c r="C7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="5" t="s">
@@ -1343,27 +1504,29 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="216.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="H8" s="1"/>
+      <c r="H8" s="1" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -1383,27 +1546,29 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="216.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" ht="216.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="F9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="H9" s="1"/>
+      <c r="H9" s="1" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -1423,7 +1588,7 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="189" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" ht="189" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="5" t="s">
         <v>28</v>
@@ -1464,7 +1629,7 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="189" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" ht="189" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="5" t="s">
         <v>33</v>
@@ -1505,7 +1670,7 @@
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
     </row>
-    <row r="12" spans="1:26" ht="168.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" ht="168.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="5" t="s">
         <v>39</v>
@@ -1547,7 +1712,7 @@
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
     </row>
-    <row r="13" spans="1:26" ht="164.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" ht="164.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="5" t="s">
         <v>44</v>
@@ -1589,18 +1754,18 @@
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
     </row>
-    <row r="14" spans="1:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="12"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="14"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -1610,27 +1775,29 @@
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
     </row>
-    <row r="15" spans="1:26" ht="240" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" ht="240" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="H15" s="8"/>
+      <c r="H15" s="8" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -1641,27 +1808,29 @@
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
     </row>
-    <row r="16" spans="1:26" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="G16" s="16" t="s">
+      <c r="G16" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="H16" s="8"/>
+      <c r="H16" s="8" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1672,25 +1841,27 @@
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
     </row>
-    <row r="17" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="11" t="s">
         <v>55</v>
       </c>
       <c r="F17" s="8"/>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="8"/>
+      <c r="H17" s="8" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -1701,23 +1872,25 @@
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
     </row>
-    <row r="18" spans="1:17" ht="258" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" ht="258" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="11" t="s">
         <v>70</v>
       </c>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
-      <c r="G18" s="16" t="s">
+      <c r="G18" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H18" s="8"/>
+      <c r="H18" s="8" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -1728,7 +1901,7 @@
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
     </row>
-    <row r="19" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1747,7 +1920,7 @@
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
     </row>
-    <row r="20" spans="1:17" ht="213.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" ht="213.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1766,7 +1939,7 @@
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
     </row>
-    <row r="21" spans="1:17" ht="213.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" ht="213.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1785,7 +1958,7 @@
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
     </row>
-    <row r="22" spans="1:17" ht="199.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" ht="199.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1804,7 +1977,7 @@
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
     </row>
-    <row r="23" spans="1:17" ht="217.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" ht="217.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1823,7 +1996,7 @@
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
     </row>
-    <row r="24" spans="1:17" ht="192.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" ht="192.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1842,7 +2015,7 @@
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
     </row>
-    <row r="25" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1861,7 +2034,7 @@
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
     </row>
-    <row r="26" spans="1:17" ht="240.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" ht="240.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1880,7 +2053,7 @@
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
     </row>
-    <row r="27" spans="1:17" ht="240.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" ht="240.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1899,7 +2072,7 @@
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
     </row>
-    <row r="28" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1918,7 +2091,7 @@
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
     </row>
-    <row r="29" spans="1:17" ht="210" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1937,7 +2110,7 @@
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
     </row>
-    <row r="30" spans="1:17" ht="276.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" ht="276.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1956,7 +2129,7 @@
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
     </row>
-    <row r="31" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1975,7 +2148,7 @@
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
     </row>
-    <row r="32" spans="1:17" ht="230.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" ht="230.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1994,7 +2167,7 @@
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33" spans="1:17" ht="230.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" ht="230.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2013,7 +2186,7 @@
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
     </row>
-    <row r="34" spans="1:17" ht="230.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" ht="230.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2032,7 +2205,7 @@
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
     </row>
-    <row r="35" spans="1:17" ht="184.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" ht="184.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2051,7 +2224,7 @@
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
     </row>
-    <row r="36" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2070,7 +2243,7 @@
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
     </row>
-    <row r="37" spans="1:17" ht="287.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" ht="287.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2089,7 +2262,7 @@
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
     </row>
-    <row r="38" spans="1:17" ht="258.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" ht="258.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2108,7 +2281,7 @@
       <c r="P38" s="1"/>
       <c r="Q38" s="1"/>
     </row>
-    <row r="39" spans="1:17" ht="258.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" ht="258.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2127,7 +2300,7 @@
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
     </row>
-    <row r="40" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2146,7 +2319,7 @@
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
     </row>
-    <row r="41" spans="1:17" ht="188.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:17" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2165,7 +2338,7 @@
       <c r="P41" s="1"/>
       <c r="Q41" s="1"/>
     </row>
-    <row r="42" spans="1:17" ht="255" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:17" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2184,7 +2357,7 @@
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
     </row>
-    <row r="43" spans="1:17" ht="158.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" ht="158.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2203,7 +2376,7 @@
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
     </row>
-    <row r="44" spans="1:17" ht="183" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:17" ht="183" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2222,7 +2395,7 @@
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
     </row>
-    <row r="45" spans="1:17" ht="183" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:17" ht="183" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2241,7 +2414,7 @@
       <c r="P45" s="1"/>
       <c r="Q45" s="1"/>
     </row>
-    <row r="46" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2260,7 +2433,7 @@
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
     </row>
-    <row r="47" spans="1:17" ht="251.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:17" ht="251.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -2279,7 +2452,7 @@
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
     </row>
-    <row r="48" spans="1:17" ht="195" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:17" ht="195" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -2298,7 +2471,7 @@
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
     </row>
-    <row r="49" spans="1:17" ht="195" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" ht="195" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -2317,7 +2490,7 @@
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
     </row>
-    <row r="50" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -2336,7 +2509,7 @@
       <c r="P50" s="1"/>
       <c r="Q50" s="1"/>
     </row>
-    <row r="51" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -2355,7 +2528,7 @@
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
     </row>
-    <row r="52" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -2374,7 +2547,7 @@
       <c r="P52" s="1"/>
       <c r="Q52" s="1"/>
     </row>
-    <row r="53" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -2393,7 +2566,7 @@
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
     </row>
-    <row r="54" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -2412,7 +2585,7 @@
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
     </row>
-    <row r="55" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -2431,7 +2604,7 @@
       <c r="P55" s="1"/>
       <c r="Q55" s="1"/>
     </row>
-    <row r="56" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -2450,7 +2623,7 @@
       <c r="P56" s="1"/>
       <c r="Q56" s="1"/>
     </row>
-    <row r="57" spans="1:17" ht="251.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" ht="251.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -2469,7 +2642,7 @@
       <c r="P57" s="1"/>
       <c r="Q57" s="1"/>
     </row>
-    <row r="58" spans="1:17" ht="251.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" ht="251.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -2488,7 +2661,7 @@
       <c r="P58" s="1"/>
       <c r="Q58" s="1"/>
     </row>
-    <row r="59" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
@@ -2507,7 +2680,7 @@
       <c r="P59" s="1"/>
       <c r="Q59" s="1"/>
     </row>
-    <row r="60" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
@@ -2526,7 +2699,7 @@
       <c r="P60" s="1"/>
       <c r="Q60" s="1"/>
     </row>
-    <row r="61" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
@@ -2545,7 +2718,7 @@
       <c r="P61" s="1"/>
       <c r="Q61" s="1"/>
     </row>
-    <row r="62" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
@@ -2564,7 +2737,7 @@
       <c r="P62" s="1"/>
       <c r="Q62" s="1"/>
     </row>
-    <row r="63" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
@@ -2583,7 +2756,7 @@
       <c r="P63" s="1"/>
       <c r="Q63" s="1"/>
     </row>
-    <row r="64" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
@@ -2602,7 +2775,7 @@
       <c r="P64" s="1"/>
       <c r="Q64" s="1"/>
     </row>
-    <row r="65" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
@@ -2621,7 +2794,7 @@
       <c r="P65" s="1"/>
       <c r="Q65" s="1"/>
     </row>
-    <row r="66" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" ht="250.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
       <c r="C66" s="1"/>

</xml_diff>